<commit_message>
fix: revertir precios Imprimador a Lista-13 (error en Lista-14)
250 ML $18.767→$11.401 | 1 Lts $36.662→$27.612 | 4 Lts $215.219→$105.669

Co-Authored-By: Claude Sonnet 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downloads/lista-precios.xlsx
+++ b/downloads/lista-precios.xlsx
@@ -5787,7 +5787,7 @@
       </ns0:c>
       <ns0:c r="C104" s="6" t="inlineStr">
         <ns0:is>
-          <ns0:t>$ 18.767</ns0:t>
+          <ns0:t>$ 11.401</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D104" s="7"/>
@@ -5801,7 +5801,7 @@
       </ns0:c>
       <ns0:c r="C105" s="6" t="inlineStr">
         <ns0:is>
-          <ns0:t>$ 36.662</ns0:t>
+          <ns0:t>$ 27.612</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D105" s="7"/>
@@ -5815,7 +5815,7 @@
       </ns0:c>
       <ns0:c r="C106" s="6" t="inlineStr">
         <ns0:is>
-          <ns0:t>$ 215.219</ns0:t>
+          <ns0:t>$ 105.669</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D106" s="7"/>

</xml_diff>

<commit_message>
fix: precios Flexible Gas Aprobado Extensibles x 3/4"
20 a 45 cm $1.441→$16.887 | 40 a 99 cm $2.137→$26.638

Co-Authored-By: Claude Sonnet 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downloads/lista-precios.xlsx
+++ b/downloads/lista-precios.xlsx
@@ -4807,7 +4807,7 @@
       </ns0:c>
       <ns0:c r="C32" s="6" t="inlineStr">
         <ns0:is>
-          <ns0:t>$ 1.441</ns0:t>
+          <ns0:t>$ 16.887</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D32" s="7"/>
@@ -4821,7 +4821,7 @@
       </ns0:c>
       <ns0:c r="C33" s="6" t="inlineStr">
         <ns0:is>
-          <ns0:t>$ 2.137</ns0:t>
+          <ns0:t>$ 26.638</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D33" s="7"/>

</xml_diff>